<commit_message>
adjustment on the account creation
</commit_message>
<xml_diff>
--- a/outputs/patient-accounts/cliniq-patient-account-import.xlsx
+++ b/outputs/patient-accounts/cliniq-patient-account-import.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Patient Accounts" sheetId="1" r:id="Rcb41609010de4f41"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="2" r:id="R8dac5bfb6a8d42ad"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Patient Accounts" sheetId="1" r:id="R8aec555f541b40b4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="2" r:id="R65e0ca81cafd4580"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -505,7 +505,7 @@
     <x:col min="4" max="4" width="18" hidden="0" customWidth="1"/>
     <x:col min="5" max="5" width="18" hidden="0" customWidth="1"/>
     <x:col min="6" max="6" width="14" hidden="0" customWidth="1"/>
-    <x:col min="7" max="7" width="27" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="32" hidden="0" customWidth="1"/>
     <x:col min="8" max="8" width="27" hidden="0" customWidth="1"/>
     <x:col min="9" max="9" width="27" hidden="0" customWidth="1"/>
     <x:col min="10" max="10" width="27" hidden="0" customWidth="1"/>
@@ -531,13 +531,13 @@
         <x:v>Birthdate</x:v>
       </x:c>
       <x:c r="G1" s="10" t="str">
-        <x:v>Program or Department</x:v>
+        <x:v>Program Code / Department or Office</x:v>
       </x:c>
       <x:c r="H1" s="10" t="str">
-        <x:v>Year Level or Employment Type</x:v>
+        <x:v>Year Level / Employment Type</x:v>
       </x:c>
       <x:c r="I1" s="10" t="str">
-        <x:v>Section or Position</x:v>
+        <x:v>Section Code / Title / Position</x:v>
       </x:c>
       <x:c r="J1" s="11" t="str">
         <x:v>Academic Year</x:v>
@@ -1746,7 +1746,7 @@
   </x:sheetData>
   <x:dataValidations count="1">
     <x:dataValidation type="list" sqref="B2:B101">
-      <x:formula1>"student,faculty,patient"</x:formula1>
+      <x:formula1>"student,faculty,school personnel"</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1792,7 +1792,7 @@
         <x:v>ID Number</x:v>
       </x:c>
       <x:c r="B5" s="36" t="str">
-        <x:v>Required. Keep leading zeroes and hyphens exactly as issued.</x:v>
+        <x:v>Required. IDs are stored in uppercase; keep leading zeroes and hyphens exactly as issued.</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -1800,7 +1800,7 @@
         <x:v>Patient Type</x:v>
       </x:c>
       <x:c r="B6" s="36" t="str">
-        <x:v>Required: student, faculty, or patient.</x:v>
+        <x:v>Required: student, faculty, or school personnel.</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -1824,39 +1824,47 @@
         <x:v>Student details</x:v>
       </x:c>
       <x:c r="B9" s="36" t="str">
-        <x:v>Use Program, Year Level, Section, and Academic Year.</x:v>
+        <x:v>Use an uppercase Program Code such as BSIT, Year Level 1 to 4, and Section Code A to E. CLINiQ stores the combined Section, for example BSIT 3 D.</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
-      <x:c r="A10" s="37" t="str">
+      <x:c r="A10" s="36" t="str">
         <x:v>Faculty details</x:v>
       </x:c>
-      <x:c r="B10" s="37" t="str">
-        <x:v>Use Department, Employment Type, and Position.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="12">
-      <x:c r="A12" s="51" t="str">
-        <x:v>Temporary passwords are generated by CLINiQ after import using the last three ID digits repeated twice. Do not add passwords to this workbook.</x:v>
-      </x:c>
-      <x:c r="B12" s="52"/>
-      <x:c r="C12" s="52"/>
-      <x:c r="D12" s="52"/>
-      <x:c r="E12" s="52"/>
-      <x:c r="F12" s="53"/>
+      <x:c r="B10" s="36" t="str">
+        <x:v>Use Department, Employment Type (Full-time or Part-time), and Title (for example DIT or MIT). Faculty titles are stored in uppercase.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11">
+      <x:c r="A11" s="37" t="str">
+        <x:v>School personnel details</x:v>
+      </x:c>
+      <x:c r="B11" s="37" t="str">
+        <x:v>Use Department or Office, Employment Type, and Position.</x:v>
+      </x:c>
     </x:row>
     <x:row r="13">
-      <x:c r="A13" s="54"/>
-      <x:c r="B13" s="55"/>
-      <x:c r="C13" s="55"/>
-      <x:c r="D13" s="55"/>
-      <x:c r="E13" s="55"/>
-      <x:c r="F13" s="56"/>
+      <x:c r="A13" s="51" t="str">
+        <x:v>Passwords are generated by CLINiQ after import using the last three ID digits repeated twice. Do not add passwords to this workbook.</x:v>
+      </x:c>
+      <x:c r="B13" s="52"/>
+      <x:c r="C13" s="52"/>
+      <x:c r="D13" s="52"/>
+      <x:c r="E13" s="52"/>
+      <x:c r="F13" s="53"/>
+    </x:row>
+    <x:row r="14">
+      <x:c r="A14" s="54"/>
+      <x:c r="B14" s="55"/>
+      <x:c r="C14" s="55"/>
+      <x:c r="D14" s="55"/>
+      <x:c r="E14" s="55"/>
+      <x:c r="F14" s="56"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:F1"/>
-    <x:mergeCell ref="A12:F13"/>
+    <x:mergeCell ref="A13:F14"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>